<commit_message>
generated 3 sheets with script
</commit_message>
<xml_diff>
--- a/static/auto_sheets/field_sample_internal.xlsx
+++ b/static/auto_sheets/field_sample_internal.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,23 +425,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>column_name</t>
+          <t>Column Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>data_type</t>
+          <t>Data Type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ordinal_position</t>
+          <t>Is Nullable</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Example data 1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Example data 2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Example data 3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Accepted format</t>
         </is>
       </c>
     </row>
@@ -456,8 +476,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>jkl223_hollerup_20230914_1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>jkl223_hollerup_20230914_2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>jkl223_hollerup_20230914_3</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>&lt;ku-id&gt;_&lt;sampling_site&gt;_&lt;sampling_date&gt;_&lt;no&gt;</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -471,9 +513,15 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -486,8 +534,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>3</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Greenland</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -501,8 +571,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>4</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -516,8 +608,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>5</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -531,8 +645,24 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>6</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="E7" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="F7" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>decimal degrees, max 2 digits, max 8 decimal points (-90 to 90)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -546,8 +676,24 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>7</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>decimal degrees, max 2 digits, max 8 decimal points (-180 to 180)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -561,8 +707,30 @@
           <t>date</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>8</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -576,8 +744,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>9</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>hlj234; glj523</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>KU Ids</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -591,8 +781,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>10</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>KU Id</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -606,8 +818,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>11</v>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NOVO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NOVO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NOVO</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -621,8 +855,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>12</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Traversing European Coastlines</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Arctic Canada</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Arctic Canada</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -636,8 +892,26 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>13</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>200</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -651,8 +925,30 @@
           <t>int4range</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>14</v>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>[10, 50)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>[10, 20)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>[-10, -5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Restricted mathematical notation of the form [&lt;no&gt;, &lt;no&gt;). Meaning only use "[" as the opening bracket and ")" as the closing bracket (decimals not allowed).</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -666,8 +962,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>15</v>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>msl</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>local surface</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CGG_3_000002</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -681,8 +999,26 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>16</v>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -696,8 +1032,26 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>17</v>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" t="n">
+        <v>200</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -711,8 +1065,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>18</v>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Monolith</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>OSL</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Mathematical notation: Numbers, "()", "[]" and "," (decimal allowed only if "." is used as decimal point).</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -726,8 +1102,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>19</v>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Lacustrine</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Glaciofluvial</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Glaciofluvial</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -741,8 +1139,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C21" t="n">
-        <v>20</v>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Outcrop</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Cave</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Lake</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -756,8 +1176,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>21</v>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -771,8 +1213,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>22</v>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Holocene</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Holocene</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Pleistocene</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Full names seperated by comma</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -786,8 +1250,30 @@
           <t>int4range</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>23</v>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>[1, 105)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>[1, 105)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>[1, 105)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Restricted mathematical notation of the form [&lt;no&gt;, &lt;no&gt;). Meaning only use "[" as the opening bracket and ")" as the closing bracket (decimals not allowed).</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -801,8 +1287,26 @@
           <t>double precision</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>24</v>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>37</v>
+      </c>
+      <c r="E25" t="n">
+        <v>37</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>37.5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Number (decimal allowed)</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -816,8 +1320,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C26" t="n">
-        <v>25</v>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Address </t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -831,8 +1357,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C27" t="n">
-        <v>26</v>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Cold room</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Walk-in Freezer</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Cold room</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -846,8 +1394,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C28" t="n">
-        <v>27</v>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -861,8 +1431,30 @@
           <t>date</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>28</v>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -876,8 +1468,30 @@
           <t>date</t>
         </is>
       </c>
-      <c r="C30" t="n">
-        <v>29</v>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -891,8 +1505,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>30</v>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water content: 10 %; </t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>water content: 10 %;</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>water content: 10 %; porosity: 5 %</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -906,8 +1542,30 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C32" t="n">
-        <v>31</v>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>temperature: 7 celcius; cloud cover: overcast;</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -921,8 +1579,18 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C33" t="n">
-        <v>32</v>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -936,8 +1604,18 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C34" t="n">
-        <v>33</v>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -951,53 +1629,18 @@
           <t>text</t>
         </is>
       </c>
-      <c r="C35" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>database_insert_by</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>from_spreadsheet</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>database_insert_datetime_utc</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>timestamp with time zone</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>37</v>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>text and/or numbers</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>